<commit_message>
Add Colab CUDA comparison results
</commit_message>
<xml_diff>
--- a/developer/fall-26/metal/cifar10_benchmark_statistics.xlsx
+++ b/developer/fall-26/metal/cifar10_benchmark_statistics.xlsx
@@ -8,17 +8,19 @@
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Inference" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="MPS vs CPU" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Training step" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="CIFAR status" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="CIFAR training" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Inference" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Throughput comparison" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Training step" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Status" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Overview'!$A$1:$B$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Inference'!$A$1:$F$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'MPS vs CPU'!$A$1:$G$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Training step'!$A$1:$F$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'CIFAR status'!$A$1:$D$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Overview'!$A$1:$B$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CIFAR training'!$A$1:$E$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Inference'!$A$1:$G$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Throughput comparison'!$A$1:$G$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Training step'!$A$1:$G$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Status'!$A$1:$E$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -26,9 +28,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="0.000"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -72,7 +72,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -438,11 +438,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="33" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -465,67 +465,67 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-21T02:44:44+05:00</t>
+          <t>2026-09-21T02:48:39+05:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Selected backend</t>
+          <t>CUDA device</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>mps (Apple Metal / MPS)</t>
+          <t>NVIDIA Tesla T4 (Google Colab)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Platform</t>
+          <t>MPS device</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>macOS-26.2-arm64-arm-64bit</t>
+          <t>Apple Metal / MPS (Mac)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>CPU baselines</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>3.12.14</t>
+          <t>Mac CPU and Colab CPU</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>PyTorch</t>
+          <t>CUDA PyTorch</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2.14.0</t>
+          <t>2.11.0+cu128</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>torchvision</t>
+          <t>MPS/CPU PyTorch</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0.29.0</t>
+          <t>2.14.0</t>
         </is>
       </c>
     </row>
@@ -566,49 +566,27 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>MPS built</t>
-        </is>
-      </c>
-      <c r="B11" t="b">
-        <v>1</v>
+          <t>CUDA final test accuracy</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0.7682</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>MPS available</t>
-        </is>
-      </c>
-      <c r="B12" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>CUDA status</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Unavailable on this Mac; run in Colab</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>CIFAR-10 accuracy status</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Pending dataset download</t>
+          <t>MPS test accuracy</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Pending local CIFAR-10 download</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B14"/>
+  <autoFilter ref="A1:B12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -619,227 +597,130 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="7" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Backend</t>
+          <t>epoch</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>batch_size</t>
+          <t>train_loss</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>mean_latency_ms</t>
+          <t>train_accuracy</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>p50_latency_ms</t>
+          <t>train_images_per_second</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>p95_latency_ms</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>throughput_images_per_second</t>
+          <t>test_accuracy</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>MPS</t>
-        </is>
+      <c r="A2" t="n">
+        <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>1</v>
+        <v>1.3089</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>1.027473328867927</v>
-      </c>
-      <c r="D2" s="2" t="n">
-        <v>1.009520958177745</v>
+        <v>0.5252</v>
+      </c>
+      <c r="D2" t="n">
+        <v>2191.9</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>1.143918483285233</v>
-      </c>
-      <c r="F2" s="2" t="n">
-        <v>973.2612729731901</v>
+        <v>0.5606</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>MPS</t>
-        </is>
+      <c r="A3" t="n">
+        <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>8</v>
+        <v>0.9282</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>1.46923825959675</v>
-      </c>
-      <c r="D3" s="2" t="n">
-        <v>1.409229007549584</v>
+        <v>0.6701</v>
+      </c>
+      <c r="D3" t="n">
+        <v>2788.6</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>1.727774803293869</v>
-      </c>
-      <c r="F3" s="2" t="n">
-        <v>5444.998418565342</v>
+        <v>0.6382</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>MPS</t>
-        </is>
+      <c r="A4" t="n">
+        <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>32</v>
+        <v>0.7783</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>3.789123818278313</v>
-      </c>
-      <c r="D4" s="2" t="n">
-        <v>3.767750051338226</v>
+        <v>0.7288</v>
+      </c>
+      <c r="D4" t="n">
+        <v>2756.2</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>3.910620824899524</v>
-      </c>
-      <c r="F4" s="2" t="n">
-        <v>8445.224155947491</v>
+        <v>0.7112000000000001</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>MPS</t>
-        </is>
+      <c r="A5" t="n">
+        <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>128</v>
+        <v>0.6778</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>14.46789498091675</v>
-      </c>
-      <c r="D5" s="2" t="n">
-        <v>14.16427048388869</v>
+        <v>0.7662</v>
+      </c>
+      <c r="D5" t="n">
+        <v>2627.6</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>16.26776050543413</v>
-      </c>
-      <c r="F5" s="2" t="n">
-        <v>8847.17508447724</v>
+        <v>0.7179</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>CPU</t>
-        </is>
+      <c r="A6" t="n">
+        <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>0.6088</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>1.145806608255953</v>
-      </c>
-      <c r="D6" s="2" t="n">
-        <v>1.143687521107495</v>
+        <v>0.7891</v>
+      </c>
+      <c r="D6" t="n">
+        <v>2710.2</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>1.345437142299488</v>
-      </c>
-      <c r="F6" s="2" t="n">
-        <v>872.7476284345341</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>CPU</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>8</v>
-      </c>
-      <c r="C7" s="2" t="n">
-        <v>4.472170085646212</v>
-      </c>
-      <c r="D7" s="2" t="n">
-        <v>4.244813055265695</v>
-      </c>
-      <c r="E7" s="2" t="n">
-        <v>5.307681573322042</v>
-      </c>
-      <c r="F7" s="2" t="n">
-        <v>1788.84072984537</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>CPU</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>32</v>
-      </c>
-      <c r="C8" s="2" t="n">
-        <v>49.55716577358544</v>
-      </c>
-      <c r="D8" s="2" t="n">
-        <v>47.83795849652961</v>
-      </c>
-      <c r="E8" s="2" t="n">
-        <v>57.14742891141213</v>
-      </c>
-      <c r="F8" s="2" t="n">
-        <v>645.7189288467417</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>CPU</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>128</v>
-      </c>
-      <c r="C9" s="2" t="n">
-        <v>105.3631699807011</v>
-      </c>
-      <c r="D9" s="2" t="n">
-        <v>97.81729202950373</v>
-      </c>
-      <c r="E9" s="2" t="n">
-        <v>142.1562545117922</v>
-      </c>
-      <c r="F9" s="2" t="n">
-        <v>1214.845757046274</v>
+        <v>0.7682</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F9"/>
+  <autoFilter ref="A1:E6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -850,149 +731,489 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="1" max="1"/>
     <col width="23" customWidth="1" min="2" max="2"/>
-    <col width="23" customWidth="1" min="3" max="3"/>
-    <col width="27" customWidth="1" min="4" max="4"/>
-    <col width="27" customWidth="1" min="5" max="5"/>
-    <col width="27" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
     <col width="30" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Batch size</t>
+          <t>Backend</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>MPS mean latency (ms)</t>
+          <t>Device</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>CPU mean latency (ms)</t>
+          <t>batch_size</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>MPS latency advantage (x)</t>
+          <t>mean_latency_ms</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>MPS throughput (images/s)</t>
+          <t>p50_latency_ms</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>CPU throughput (images/s)</t>
+          <t>p95_latency_ms</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>MPS throughput advantage (x)</t>
+          <t>throughput_images_per_second</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>CUDA</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Google Colab Tesla T4</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="n">
+      <c r="D2" t="n">
+        <v>0.646</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.638</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.714</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1546.9</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>CUDA</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Google Colab Tesla T4</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>8</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.905</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1.025</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1.061</v>
+      </c>
+      <c r="G3" t="n">
+        <v>8837.299999999999</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>CUDA</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Google Colab Tesla T4</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>32</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1.79</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1.779</v>
+      </c>
+      <c r="F4" t="n">
+        <v>1.877</v>
+      </c>
+      <c r="G4" t="n">
+        <v>17877.3</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>CUDA</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Google Colab Tesla T4</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>128</v>
+      </c>
+      <c r="D5" t="n">
+        <v>6.67</v>
+      </c>
+      <c r="E5" t="n">
+        <v>6.64</v>
+      </c>
+      <c r="F5" t="n">
+        <v>6.716</v>
+      </c>
+      <c r="G5" t="n">
+        <v>19189.5</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>MPS</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Mac Apple Metal / MPS</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="n">
         <v>1.027473328867927</v>
       </c>
-      <c r="C2" s="2" t="n">
+      <c r="E6" t="n">
+        <v>1.009520958177745</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1.143918483285233</v>
+      </c>
+      <c r="G6" t="n">
+        <v>973.2612729731901</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>MPS</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Mac Apple Metal / MPS</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>8</v>
+      </c>
+      <c r="D7" t="n">
+        <v>1.46923825959675</v>
+      </c>
+      <c r="E7" t="n">
+        <v>1.409229007549584</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1.727774803293869</v>
+      </c>
+      <c r="G7" t="n">
+        <v>5444.998418565342</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>MPS</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Mac Apple Metal / MPS</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>32</v>
+      </c>
+      <c r="D8" t="n">
+        <v>3.789123818278313</v>
+      </c>
+      <c r="E8" t="n">
+        <v>3.767750051338226</v>
+      </c>
+      <c r="F8" t="n">
+        <v>3.910620824899524</v>
+      </c>
+      <c r="G8" t="n">
+        <v>8445.224155947491</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>MPS</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Mac Apple Metal / MPS</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>128</v>
+      </c>
+      <c r="D9" t="n">
+        <v>14.46789498091675</v>
+      </c>
+      <c r="E9" t="n">
+        <v>14.16427048388869</v>
+      </c>
+      <c r="F9" t="n">
+        <v>16.26776050543413</v>
+      </c>
+      <c r="G9" t="n">
+        <v>8847.17508447724</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Mac CPU</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" t="n">
         <v>1.145806608255953</v>
       </c>
-      <c r="D2" s="2" t="n">
-        <v>1.115169198132282</v>
-      </c>
-      <c r="E2" s="2" t="n">
-        <v>973.2612729731901</v>
-      </c>
-      <c r="F2" s="2" t="n">
+      <c r="E10" t="n">
+        <v>1.143687521107495</v>
+      </c>
+      <c r="F10" t="n">
+        <v>1.345437142299488</v>
+      </c>
+      <c r="G10" t="n">
         <v>872.7476284345341</v>
       </c>
-      <c r="G2" s="2" t="n">
-        <v>1.115169198132282</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Mac CPU</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
         <v>8</v>
       </c>
-      <c r="B3" s="2" t="n">
-        <v>1.46923825959675</v>
-      </c>
-      <c r="C3" s="2" t="n">
+      <c r="D11" t="n">
         <v>4.472170085646212</v>
       </c>
-      <c r="D3" s="2" t="n">
-        <v>3.043869880487357</v>
-      </c>
-      <c r="E3" s="2" t="n">
-        <v>5444.998418565342</v>
-      </c>
-      <c r="F3" s="2" t="n">
+      <c r="E11" t="n">
+        <v>4.244813055265695</v>
+      </c>
+      <c r="F11" t="n">
+        <v>5.307681573322042</v>
+      </c>
+      <c r="G11" t="n">
         <v>1788.84072984537</v>
       </c>
-      <c r="G3" s="2" t="n">
-        <v>3.043869880487357</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Mac CPU</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
         <v>32</v>
       </c>
-      <c r="B4" s="2" t="n">
-        <v>3.789123818278313</v>
-      </c>
-      <c r="C4" s="2" t="n">
+      <c r="D12" t="n">
         <v>49.55716577358544</v>
       </c>
-      <c r="D4" s="2" t="n">
-        <v>13.07879292160556</v>
-      </c>
-      <c r="E4" s="2" t="n">
-        <v>8445.224155947491</v>
-      </c>
-      <c r="F4" s="2" t="n">
+      <c r="E12" t="n">
+        <v>47.83795849652961</v>
+      </c>
+      <c r="F12" t="n">
+        <v>57.14742891141213</v>
+      </c>
+      <c r="G12" t="n">
         <v>645.7189288467417</v>
       </c>
-      <c r="G4" s="2" t="n">
-        <v>13.07879292160556</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Mac CPU</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
         <v>128</v>
       </c>
-      <c r="B5" s="2" t="n">
-        <v>14.46789498091675</v>
-      </c>
-      <c r="C5" s="2" t="n">
+      <c r="D13" t="n">
         <v>105.3631699807011</v>
       </c>
-      <c r="D5" s="2" t="n">
-        <v>7.282550095896864</v>
-      </c>
-      <c r="E5" s="2" t="n">
-        <v>8847.17508447724</v>
-      </c>
-      <c r="F5" s="2" t="n">
+      <c r="E13" t="n">
+        <v>97.81729202950373</v>
+      </c>
+      <c r="F13" t="n">
+        <v>142.1562545117922</v>
+      </c>
+      <c r="G13" t="n">
         <v>1214.845757046274</v>
       </c>
-      <c r="G5" s="2" t="n">
-        <v>7.282550095896864</v>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Colab CPU</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" t="n">
+        <v>4.021</v>
+      </c>
+      <c r="E14" t="n">
+        <v>3.827</v>
+      </c>
+      <c r="F14" t="n">
+        <v>5.599</v>
+      </c>
+      <c r="G14" t="n">
+        <v>248.7</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Colab CPU</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>8</v>
+      </c>
+      <c r="D15" t="n">
+        <v>22.733</v>
+      </c>
+      <c r="E15" t="n">
+        <v>22.222</v>
+      </c>
+      <c r="F15" t="n">
+        <v>27.027</v>
+      </c>
+      <c r="G15" t="n">
+        <v>351.9</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Colab CPU</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>32</v>
+      </c>
+      <c r="D16" t="n">
+        <v>95.748</v>
+      </c>
+      <c r="E16" t="n">
+        <v>86.34699999999999</v>
+      </c>
+      <c r="F16" t="n">
+        <v>132.7</v>
+      </c>
+      <c r="G16" t="n">
+        <v>334.2</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Colab CPU</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>128</v>
+      </c>
+      <c r="D17" t="n">
+        <v>481.498</v>
+      </c>
+      <c r="E17" t="n">
+        <v>462.027</v>
+      </c>
+      <c r="F17" t="n">
+        <v>659.143</v>
+      </c>
+      <c r="G17" t="n">
+        <v>265.8</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G5"/>
+  <autoFilter ref="A1:G17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1003,113 +1224,149 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="21" customWidth="1" min="3" max="3"/>
-    <col width="19" customWidth="1" min="4" max="4"/>
-    <col width="19" customWidth="1" min="5" max="5"/>
-    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="27" customWidth="1" min="3" max="3"/>
+    <col width="31" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="23" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Backend</t>
+          <t>Batch size</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>batch_size</t>
+          <t>CUDA throughput (images/s)</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>mean_step_ms</t>
+          <t>MPS throughput (images/s)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>p50_step_ms</t>
+          <t>Mac CPU throughput (images/s)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>p95_step_ms</t>
+          <t>CUDA vs MPS (x)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>training_images_per_second</t>
+          <t>MPS vs Mac CPU (x)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>CUDA vs Colab CPU (x)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>MPS</t>
-        </is>
+      <c r="A2" t="n">
+        <v>1</v>
       </c>
       <c r="B2" t="n">
+        <v>1546.9</v>
+      </c>
+      <c r="C2" t="n">
+        <v>973.2612729731901</v>
+      </c>
+      <c r="D2" t="n">
+        <v>872.7476284345341</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1.589398492425797</v>
+      </c>
+      <c r="F2" t="n">
+        <v>1.115169198132282</v>
+      </c>
+      <c r="G2" t="n">
+        <v>6.219943707277846</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B3" t="n">
+        <v>8837.299999999999</v>
+      </c>
+      <c r="C3" t="n">
+        <v>5444.998418565342</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1788.84072984537</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1.623012408941795</v>
+      </c>
+      <c r="F3" t="n">
+        <v>3.043869880487357</v>
+      </c>
+      <c r="G3" t="n">
+        <v>25.1131003125888</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>32</v>
+      </c>
+      <c r="B4" t="n">
+        <v>17877.3</v>
+      </c>
+      <c r="C4" t="n">
+        <v>8445.224155947491</v>
+      </c>
+      <c r="D4" t="n">
+        <v>645.7189288467417</v>
+      </c>
+      <c r="E4" t="n">
+        <v>2.11685322614084</v>
+      </c>
+      <c r="F4" t="n">
+        <v>13.07879292160556</v>
+      </c>
+      <c r="G4" t="n">
+        <v>53.49281867145422</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
         <v>128</v>
       </c>
-      <c r="C2" t="n">
-        <v>40.92933754436672</v>
-      </c>
-      <c r="D2" t="n">
-        <v>40.64452101010829</v>
-      </c>
-      <c r="E2" t="n">
-        <v>41.82305230060592</v>
-      </c>
-      <c r="F2" t="n">
-        <v>3127.341112258418</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>CPU</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>128</v>
-      </c>
-      <c r="C3" t="n">
-        <v>355.561531346757</v>
-      </c>
-      <c r="D3" t="n">
-        <v>351.557687507011</v>
-      </c>
-      <c r="E3" t="n">
-        <v>377.1048767201137</v>
-      </c>
-      <c r="F3" t="n">
-        <v>359.9939496130969</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>CUDA</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>128</v>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Unavailable locally</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
+      <c r="B5" t="n">
+        <v>19189.5</v>
+      </c>
+      <c r="C5" t="n">
+        <v>8847.17508447724</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1214.845757046274</v>
+      </c>
+      <c r="E5" t="n">
+        <v>2.168997427627359</v>
+      </c>
+      <c r="F5" t="n">
+        <v>7.282550095896864</v>
+      </c>
+      <c r="G5" t="n">
+        <v>72.19525959367945</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F4"/>
+  <autoFilter ref="A1:G5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1120,13 +1377,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="29" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1137,76 +1397,238 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Training</t>
+          <t>Device</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Test accuracy</t>
+          <t>batch_size</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>mean_step_ms</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>p50_step_ms</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>p95_step_ms</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>training_images_per_second</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>MPS</t>
+          <t>CUDA</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>5 epochs pending</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Dataset download incomplete</t>
-        </is>
+          <t>Tesla T4 / Colab</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>128</v>
+      </c>
+      <c r="D2" t="n">
+        <v>22.11551510004938</v>
+      </c>
+      <c r="E2" t="n">
+        <v>22.12051499986956</v>
+      </c>
+      <c r="F2" t="n">
+        <v>22.3654986001975</v>
+      </c>
+      <c r="G2" t="n">
+        <v>5787.791937964593</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CPU</t>
+          <t>MPS</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Not run</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Synthetic baseline only</t>
-        </is>
+          <t>Apple Metal / Mac</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>128</v>
+      </c>
+      <c r="D3" t="n">
+        <v>40.92933754436672</v>
+      </c>
+      <c r="E3" t="n">
+        <v>40.64452101010829</v>
+      </c>
+      <c r="F3" t="n">
+        <v>41.82305230060592</v>
+      </c>
+      <c r="G3" t="n">
+        <v>3127.341112258418</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>CPU</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Mac CPU</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>128</v>
+      </c>
+      <c r="D4" t="n">
+        <v>355.561531346757</v>
+      </c>
+      <c r="E4" t="n">
+        <v>351.557687507011</v>
+      </c>
+      <c r="F4" t="n">
+        <v>377.1048767201137</v>
+      </c>
+      <c r="G4" t="n">
+        <v>359.9939496130969</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G4"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Device</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Training status</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Test accuracy</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
           <t>CUDA</t>
         </is>
       </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Tesla T4 / Colab</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Completed 5 epochs</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>0.7682</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Measured in cifar10_cuda_google_collab.ipynb</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>MPS</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Apple Metal / Mac</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Pending dataset completion</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>MPS operation and synthetic benchmarks verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>CPU</t>
+        </is>
+      </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Not run locally</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Run in Google Colab</t>
+          <t>Mac CPU</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Synthetic baseline only</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Same architecture/weights for inference</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D4"/>
+  <autoFilter ref="A1:E4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Record completed MPS CIFAR results
</commit_message>
<xml_diff>
--- a/developer/fall-26/metal/cifar10_benchmark_statistics.xlsx
+++ b/developer/fall-26/metal/cifar10_benchmark_statistics.xlsx
@@ -8,19 +8,17 @@
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="CIFAR training" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Training epochs" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Inference" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Throughput comparison" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Training step" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Status" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Overview'!$A$1:$B$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CIFAR training'!$A$1:$E$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Overview'!$A$1:$B$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Training epochs'!$A$1:$G$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Inference'!$A$1:$G$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Throughput comparison'!$A$1:$G$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Training step'!$A$1:$G$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Status'!$A$1:$E$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -438,11 +436,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="33" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -460,133 +458,83 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated</t>
+          <t>CUDA device</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-21T02:48:39+05:00</t>
+          <t>NVIDIA Tesla T4 / Google Colab</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CUDA device</t>
+          <t>MPS device</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>NVIDIA Tesla T4 (Google Colab)</t>
+          <t>Apple Metal / Mac</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>MPS device</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Apple Metal / MPS (Mac)</t>
-        </is>
+          <t>CUDA final accuracy</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0.7682</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CPU baselines</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Mac CPU and Colab CPU</t>
-        </is>
+          <t>MPS final accuracy</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0.7559999823570251</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CUDA PyTorch</t>
+          <t>Precision</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2.11.0+cu128</t>
+          <t>float32</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>MPS/CPU PyTorch</t>
+          <t>Model</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2.14.0</t>
+          <t>SmallCIFARNet</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Precision</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>float32</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Model</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>SmallCIFARNet</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Trainable parameters</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
+          <t>Parameters</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
         <v>558538</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>CUDA final test accuracy</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>0.7682</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>MPS test accuracy</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Pending local CIFAR-10 download</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:B12"/>
+  <autoFilter ref="A1:B8"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -597,130 +545,297 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="7" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>epoch</t>
+          <t>Backend</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>train_loss</t>
+          <t>Epoch</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>train_accuracy</t>
+          <t>Train loss</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>train_images_per_second</t>
+          <t>Train accuracy</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>test_accuracy</t>
+          <t>Train images/s</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Test loss</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Test accuracy</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>CUDA</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" t="n">
+      <c r="C2" t="n">
         <v>1.3089</v>
       </c>
-      <c r="C2" s="2" t="n">
+      <c r="D2" s="2" t="n">
         <v>0.5252</v>
       </c>
-      <c r="D2" t="n">
+      <c r="E2" t="n">
         <v>2191.9</v>
       </c>
-      <c r="E2" s="2" t="n">
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" s="2" t="n">
         <v>0.5606</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>CUDA</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
         <v>2</v>
       </c>
-      <c r="B3" t="n">
+      <c r="C3" t="n">
         <v>0.9282</v>
       </c>
-      <c r="C3" s="2" t="n">
+      <c r="D3" s="2" t="n">
         <v>0.6701</v>
       </c>
-      <c r="D3" t="n">
+      <c r="E3" t="n">
         <v>2788.6</v>
       </c>
-      <c r="E3" s="2" t="n">
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" s="2" t="n">
         <v>0.6382</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>CUDA</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
         <v>3</v>
       </c>
-      <c r="B4" t="n">
+      <c r="C4" t="n">
         <v>0.7783</v>
       </c>
-      <c r="C4" s="2" t="n">
+      <c r="D4" s="2" t="n">
         <v>0.7288</v>
       </c>
-      <c r="D4" t="n">
+      <c r="E4" t="n">
         <v>2756.2</v>
       </c>
-      <c r="E4" s="2" t="n">
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" s="2" t="n">
         <v>0.7112000000000001</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>CUDA</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
         <v>4</v>
       </c>
-      <c r="B5" t="n">
+      <c r="C5" t="n">
         <v>0.6778</v>
       </c>
-      <c r="C5" s="2" t="n">
+      <c r="D5" s="2" t="n">
         <v>0.7662</v>
       </c>
-      <c r="D5" t="n">
+      <c r="E5" t="n">
         <v>2627.6</v>
       </c>
-      <c r="E5" s="2" t="n">
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" s="2" t="n">
         <v>0.7179</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>CUDA</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
         <v>5</v>
       </c>
-      <c r="B6" t="n">
+      <c r="C6" t="n">
         <v>0.6088</v>
       </c>
-      <c r="C6" s="2" t="n">
+      <c r="D6" s="2" t="n">
         <v>0.7891</v>
       </c>
-      <c r="D6" t="n">
+      <c r="E6" t="n">
         <v>2710.2</v>
       </c>
-      <c r="E6" s="2" t="n">
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" s="2" t="n">
         <v>0.7682</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>MPS</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" t="n">
+        <v>1.316709637641907</v>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>0.5240399837493896</v>
+      </c>
+      <c r="E7" t="n">
+        <v>2716.90133925072</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1.377580642700195</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>0.5299999713897705</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>MPS</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>2</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0.9383672475814819</v>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>0.6691200137138367</v>
+      </c>
+      <c r="E8" t="n">
+        <v>3060.120418586794</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1.614287257194519</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>0.5167999863624573</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>MPS</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>3</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.784754753112793</v>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>0.7235000133514404</v>
+      </c>
+      <c r="E9" t="n">
+        <v>3091.729751216993</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1.029844880104065</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>0.6417999863624573</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>MPS</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>4</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0.682127833366394</v>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>0.761900007724762</v>
+      </c>
+      <c r="E10" t="n">
+        <v>3090.262193663685</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.7233282923698425</v>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>0.7480999827384949</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>MPS</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>5</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0.6103442907333374</v>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>0.7885599732398987</v>
+      </c>
+      <c r="E11" t="n">
+        <v>3093.490575032541</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.7132961750030518</v>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>0.7559999823570251</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E6"/>
+  <autoFilter ref="A1:G11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -735,7 +850,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="23" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
@@ -788,7 +903,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Google Colab Tesla T4</t>
+          <t>Tesla T4 / Google Colab</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -815,7 +930,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Google Colab Tesla T4</t>
+          <t>Tesla T4 / Google Colab</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -842,7 +957,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Google Colab Tesla T4</t>
+          <t>Tesla T4 / Google Colab</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -869,7 +984,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Google Colab Tesla T4</t>
+          <t>Tesla T4 / Google Colab</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -896,23 +1011,23 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Mac Apple Metal / MPS</t>
+          <t>Apple Metal / Mac</t>
         </is>
       </c>
       <c r="C6" t="n">
         <v>1</v>
       </c>
       <c r="D6" t="n">
-        <v>1.027473328867927</v>
+        <v>0.9820935159223154</v>
       </c>
       <c r="E6" t="n">
-        <v>1.009520958177745</v>
+        <v>0.9644374949857593</v>
       </c>
       <c r="F6" t="n">
-        <v>1.143918483285233</v>
+        <v>1.149170845746994</v>
       </c>
       <c r="G6" t="n">
-        <v>973.2612729731901</v>
+        <v>1018.232972509617</v>
       </c>
     </row>
     <row r="7">
@@ -923,23 +1038,23 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Mac Apple Metal / MPS</t>
+          <t>Apple Metal / Mac</t>
         </is>
       </c>
       <c r="C7" t="n">
         <v>8</v>
       </c>
       <c r="D7" t="n">
-        <v>1.46923825959675</v>
+        <v>1.62761832063552</v>
       </c>
       <c r="E7" t="n">
-        <v>1.409229007549584</v>
+        <v>1.54335395200178</v>
       </c>
       <c r="F7" t="n">
-        <v>1.727774803293869</v>
+        <v>2.023339859442783</v>
       </c>
       <c r="G7" t="n">
-        <v>5444.998418565342</v>
+        <v>4915.157256817016</v>
       </c>
     </row>
     <row r="8">
@@ -950,23 +1065,23 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Mac Apple Metal / MPS</t>
+          <t>Apple Metal / Mac</t>
         </is>
       </c>
       <c r="C8" t="n">
         <v>32</v>
       </c>
       <c r="D8" t="n">
-        <v>3.789123818278313</v>
+        <v>3.971538530895486</v>
       </c>
       <c r="E8" t="n">
-        <v>3.767750051338226</v>
+        <v>3.89424996683374</v>
       </c>
       <c r="F8" t="n">
-        <v>3.910620824899524</v>
+        <v>4.392377333715556</v>
       </c>
       <c r="G8" t="n">
-        <v>8445.224155947491</v>
+        <v>8057.330868393909</v>
       </c>
     </row>
     <row r="9">
@@ -977,23 +1092,23 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Mac Apple Metal / MPS</t>
+          <t>Apple Metal / Mac</t>
         </is>
       </c>
       <c r="C9" t="n">
         <v>128</v>
       </c>
       <c r="D9" t="n">
-        <v>14.46789498091675</v>
+        <v>14.07109022489749</v>
       </c>
       <c r="E9" t="n">
-        <v>14.16427048388869</v>
+        <v>14.01495799655095</v>
       </c>
       <c r="F9" t="n">
-        <v>16.26776050543413</v>
+        <v>14.59783986210823</v>
       </c>
       <c r="G9" t="n">
-        <v>8847.17508447724</v>
+        <v>9096.66542920149</v>
       </c>
     </row>
     <row r="10">
@@ -1011,16 +1126,16 @@
         <v>1</v>
       </c>
       <c r="D10" t="n">
-        <v>1.145806608255953</v>
+        <v>1.227970499312505</v>
       </c>
       <c r="E10" t="n">
-        <v>1.143687521107495</v>
+        <v>1.224583480507135</v>
       </c>
       <c r="F10" t="n">
-        <v>1.345437142299488</v>
+        <v>1.324383303290233</v>
       </c>
       <c r="G10" t="n">
-        <v>872.7476284345341</v>
+        <v>814.3518110246645</v>
       </c>
     </row>
     <row r="11">
@@ -1038,16 +1153,16 @@
         <v>8</v>
       </c>
       <c r="D11" t="n">
-        <v>4.472170085646212</v>
+        <v>4.136130405822769</v>
       </c>
       <c r="E11" t="n">
-        <v>4.244813055265695</v>
+        <v>4.058041551616043</v>
       </c>
       <c r="F11" t="n">
-        <v>5.307681573322042</v>
+        <v>4.813647555420175</v>
       </c>
       <c r="G11" t="n">
-        <v>1788.84072984537</v>
+        <v>1934.17499330721</v>
       </c>
     </row>
     <row r="12">
@@ -1065,16 +1180,16 @@
         <v>32</v>
       </c>
       <c r="D12" t="n">
-        <v>49.55716577358544</v>
+        <v>49.21745458850637</v>
       </c>
       <c r="E12" t="n">
-        <v>47.83795849652961</v>
+        <v>46.88520799390972</v>
       </c>
       <c r="F12" t="n">
-        <v>57.14742891141213</v>
+        <v>59.68016730621457</v>
       </c>
       <c r="G12" t="n">
-        <v>645.7189288467417</v>
+        <v>650.1758424433611</v>
       </c>
     </row>
     <row r="13">
@@ -1092,16 +1207,16 @@
         <v>128</v>
       </c>
       <c r="D13" t="n">
-        <v>105.3631699807011</v>
+        <v>98.52449533413164</v>
       </c>
       <c r="E13" t="n">
-        <v>97.81729202950373</v>
+        <v>95.51041648956016</v>
       </c>
       <c r="F13" t="n">
-        <v>142.1562545117922</v>
+        <v>119.3785494600888</v>
       </c>
       <c r="G13" t="n">
-        <v>1214.845757046274</v>
+        <v>1299.169303693527</v>
       </c>
     </row>
     <row r="14">
@@ -1227,49 +1342,49 @@
   <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="27" customWidth="1" min="3" max="3"/>
-    <col width="31" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="23" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Batch size</t>
+          <t>Batch</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>CUDA throughput (images/s)</t>
+          <t>CUDA img/s</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>MPS throughput (images/s)</t>
+          <t>MPS img/s</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Mac CPU throughput (images/s)</t>
+          <t>Mac CPU img/s</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>CUDA vs MPS (x)</t>
+          <t>CUDA/MPS</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>MPS vs Mac CPU (x)</t>
+          <t>MPS/Mac CPU</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>CUDA vs Colab CPU (x)</t>
+          <t>CUDA/Colab CPU</t>
         </is>
       </c>
     </row>
@@ -1281,16 +1396,16 @@
         <v>1546.9</v>
       </c>
       <c r="C2" t="n">
-        <v>973.2612729731901</v>
+        <v>1018.232972509617</v>
       </c>
       <c r="D2" t="n">
-        <v>872.7476284345341</v>
+        <v>814.3518110246645</v>
       </c>
       <c r="E2" t="n">
-        <v>1.589398492425797</v>
+        <v>1.51920045978023</v>
       </c>
       <c r="F2" t="n">
-        <v>1.115169198132282</v>
+        <v>1.25036005166909</v>
       </c>
       <c r="G2" t="n">
         <v>6.219943707277846</v>
@@ -1304,16 +1419,16 @@
         <v>8837.299999999999</v>
       </c>
       <c r="C3" t="n">
-        <v>5444.998418565342</v>
+        <v>4915.157256817016</v>
       </c>
       <c r="D3" t="n">
-        <v>1788.84072984537</v>
+        <v>1934.17499330721</v>
       </c>
       <c r="E3" t="n">
-        <v>1.623012408941795</v>
+        <v>1.797968923119035</v>
       </c>
       <c r="F3" t="n">
-        <v>3.043869880487357</v>
+        <v>2.541216422415161</v>
       </c>
       <c r="G3" t="n">
         <v>25.1131003125888</v>
@@ -1327,16 +1442,16 @@
         <v>17877.3</v>
       </c>
       <c r="C4" t="n">
-        <v>8445.224155947491</v>
+        <v>8057.330868393909</v>
       </c>
       <c r="D4" t="n">
-        <v>645.7189288467417</v>
+        <v>650.1758424433611</v>
       </c>
       <c r="E4" t="n">
-        <v>2.11685322614084</v>
+        <v>2.218762055574309</v>
       </c>
       <c r="F4" t="n">
-        <v>13.07879292160556</v>
+        <v>12.39254112874212</v>
       </c>
       <c r="G4" t="n">
         <v>53.49281867145422</v>
@@ -1350,16 +1465,16 @@
         <v>19189.5</v>
       </c>
       <c r="C5" t="n">
-        <v>8847.17508447724</v>
+        <v>9096.66542920149</v>
       </c>
       <c r="D5" t="n">
-        <v>1214.845757046274</v>
+        <v>1299.169303693527</v>
       </c>
       <c r="E5" t="n">
-        <v>2.168997427627359</v>
+        <v>2.109509264614612</v>
       </c>
       <c r="F5" t="n">
-        <v>7.282550095896864</v>
+        <v>7.001909145589991</v>
       </c>
       <c r="G5" t="n">
         <v>72.19525959367945</v>
@@ -1468,16 +1583,16 @@
         <v>128</v>
       </c>
       <c r="D3" t="n">
-        <v>40.92933754436672</v>
+        <v>43.3502273936756</v>
       </c>
       <c r="E3" t="n">
-        <v>40.64452101010829</v>
+        <v>42.44889650726691</v>
       </c>
       <c r="F3" t="n">
-        <v>41.82305230060592</v>
+        <v>48.63493127049878</v>
       </c>
       <c r="G3" t="n">
-        <v>3127.341112258418</v>
+        <v>2952.695007516247</v>
       </c>
     </row>
     <row r="4">
@@ -1495,140 +1610,20 @@
         <v>128</v>
       </c>
       <c r="D4" t="n">
-        <v>355.561531346757</v>
+        <v>356.643602498807</v>
       </c>
       <c r="E4" t="n">
-        <v>351.557687507011</v>
+        <v>352.2401250083931</v>
       </c>
       <c r="F4" t="n">
-        <v>377.1048767201137</v>
+        <v>391.4931375184096</v>
       </c>
       <c r="G4" t="n">
-        <v>359.9939496130969</v>
+        <v>358.901713372044</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:G4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="19" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Backend</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Device</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Training status</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Test accuracy</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>CUDA</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Tesla T4 / Colab</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Completed 5 epochs</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="n">
-        <v>0.7682</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Measured in cifar10_cuda_google_collab.ipynb</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>MPS</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Apple Metal / Mac</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Pending dataset completion</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>MPS operation and synthetic benchmarks verified</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>CPU</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Mac CPU</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Synthetic baseline only</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Same architecture/weights for inference</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:E4"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Add profiling results to benchmark workbook
</commit_message>
<xml_diff>
--- a/developer/fall-26/metal/cifar10_benchmark_statistics.xlsx
+++ b/developer/fall-26/metal/cifar10_benchmark_statistics.xlsx
@@ -12,6 +12,8 @@
     <sheet name="Inference" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Throughput comparison" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Training step" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Detailed profile (MPS)" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Profile comparison" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Overview'!$A$1:$B$8</definedName>
@@ -26,8 +28,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="2">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.000"/>
+  </numFmts>
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -39,8 +43,11 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -50,6 +57,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="005B9BD5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAD3"/>
       </patternFill>
     </fill>
   </fills>
@@ -65,12 +82,25 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -612,7 +642,6 @@
       <c r="E2" t="n">
         <v>2191.9</v>
       </c>
-      <c r="F2" t="inlineStr"/>
       <c r="G2" s="2" t="n">
         <v>0.5606</v>
       </c>
@@ -635,7 +664,6 @@
       <c r="E3" t="n">
         <v>2788.6</v>
       </c>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" s="2" t="n">
         <v>0.6382</v>
       </c>
@@ -658,7 +686,6 @@
       <c r="E4" t="n">
         <v>2756.2</v>
       </c>
-      <c r="F4" t="inlineStr"/>
       <c r="G4" s="2" t="n">
         <v>0.7112000000000001</v>
       </c>
@@ -681,7 +708,6 @@
       <c r="E5" t="n">
         <v>2627.6</v>
       </c>
-      <c r="F5" t="inlineStr"/>
       <c r="G5" s="2" t="n">
         <v>0.7179</v>
       </c>
@@ -704,7 +730,6 @@
       <c r="E6" t="n">
         <v>2710.2</v>
       </c>
-      <c r="F6" t="inlineStr"/>
       <c r="G6" s="2" t="n">
         <v>0.7682</v>
       </c>
@@ -1626,4 +1651,918 @@
   <autoFilter ref="A1:G4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="19" customWidth="1" min="9" max="9"/>
+    <col width="19" customWidth="1" min="10" max="10"/>
+    <col width="19" customWidth="1" min="11" max="11"/>
+    <col width="19" customWidth="1" min="12" max="12"/>
+    <col width="55" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Detailed runtime profile — Apple Metal / MPS</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>All accelerator timings are synchronized before and after each iteration. Numbers are milliseconds except throughput.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Device</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Apple Metal / MPS</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>PyTorch</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2.14.0</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Precision</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>float32</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Batch</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Input transfer mean ms</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Input transfer p50 ms</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Input transfer p95 ms</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Model mean ms</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>Model p50 ms</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>Model p95 ms</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>Model img/s</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>End-to-end mean ms</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>End-to-end p50 ms</t>
+        </is>
+      </c>
+      <c r="K5" s="5" t="inlineStr">
+        <is>
+          <t>End-to-end p95 ms</t>
+        </is>
+      </c>
+      <c r="L5" s="5" t="inlineStr">
+        <is>
+          <t>End-to-end img/s</t>
+        </is>
+      </c>
+      <c r="M5" s="5" t="inlineStr">
+        <is>
+          <t>Device timing method</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>0.189811889140401</v>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>0.1779794984031469</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>0.2395798102952539</v>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>1.214466894889483</v>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>1.077749984688126</v>
+      </c>
+      <c r="G6" s="6" t="n">
+        <v>2.05801633419469</v>
+      </c>
+      <c r="H6" s="6" t="n">
+        <v>823.4065532852587</v>
+      </c>
+      <c r="I6" s="6" t="n">
+        <v>2.516636250220472</v>
+      </c>
+      <c r="J6" s="6" t="n">
+        <v>1.948958000866696</v>
+      </c>
+      <c r="K6" s="6" t="n">
+        <v>4.343005895498208</v>
+      </c>
+      <c r="L6" s="6" t="n">
+        <v>397.3557958216624</v>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>host monotonic clock bracketed by torch.mps.synchronize()</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>8</v>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>0.3496912553964648</v>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>0.2423334954073653</v>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>0.6436497074901123</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>1.50210502644768</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>1.448062495910563</v>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>1.791173531091772</v>
+      </c>
+      <c r="H7" s="6" t="n">
+        <v>5325.859283567645</v>
+      </c>
+      <c r="I7" s="6" t="n">
+        <v>3.083426739467541</v>
+      </c>
+      <c r="J7" s="6" t="n">
+        <v>2.909833507146686</v>
+      </c>
+      <c r="K7" s="6" t="n">
+        <v>4.786495564621872</v>
+      </c>
+      <c r="L7" s="6" t="n">
+        <v>2594.515996634794</v>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>host monotonic clock bracketed by torch.mps.synchronize()</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>32</v>
+      </c>
+      <c r="B8" s="6" t="n">
+        <v>0.535589375795098</v>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>0.3377499961061403</v>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>2.087218749511521</v>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>5.689578560413793</v>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>4.981688005500473</v>
+      </c>
+      <c r="G8" s="6" t="n">
+        <v>10.12898125773063</v>
+      </c>
+      <c r="H8" s="6" t="n">
+        <v>5624.318156470397</v>
+      </c>
+      <c r="I8" s="6" t="n">
+        <v>8.676391015033005</v>
+      </c>
+      <c r="J8" s="6" t="n">
+        <v>7.612895497004502</v>
+      </c>
+      <c r="K8" s="6" t="n">
+        <v>15.66891460679471</v>
+      </c>
+      <c r="L8" s="6" t="n">
+        <v>3688.169417970644</v>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>host monotonic clock bracketed by torch.mps.synchronize()</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>128</v>
+      </c>
+      <c r="B9" s="6" t="n">
+        <v>0.3770370587881189</v>
+      </c>
+      <c r="C9" s="6" t="n">
+        <v>0.3462705062702298</v>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>0.4669496571295894</v>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>14.09337812292506</v>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>14.00985399959609</v>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>14.54687855293741</v>
+      </c>
+      <c r="H9" s="6" t="n">
+        <v>9082.279555941823</v>
+      </c>
+      <c r="I9" s="6" t="n">
+        <v>14.51253311970504</v>
+      </c>
+      <c r="J9" s="6" t="n">
+        <v>14.40779148833826</v>
+      </c>
+      <c r="K9" s="6" t="n">
+        <v>15.33372946287272</v>
+      </c>
+      <c r="L9" s="6" t="n">
+        <v>8819.962644991472</v>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>host monotonic clock bracketed by torch.mps.synchronize()</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Training step (forward + loss + backward + optimizer)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Batch</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Mean ms</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>p50 ms</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>p95 ms</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Images/s</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>Device timing method</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>128</v>
+      </c>
+      <c r="B13" s="6" t="n">
+        <v>43.31685922166798</v>
+      </c>
+      <c r="C13" s="6" t="n">
+        <v>42.16202101088129</v>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>49.91002936294535</v>
+      </c>
+      <c r="E13" s="6" t="n">
+        <v>2954.969549961549</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>host monotonic clock bracketed by torch.mps.synchronize()</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>Top MPS dispatch operators (CPU-side profiler cost; not Metal kernel duration)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Operator</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Calls</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Self CPU ms</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>CPU total ms</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>aten::native_batch_norm</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>50</v>
+      </c>
+      <c r="C17" s="6" t="n">
+        <v>8.259672000000007</v>
+      </c>
+      <c r="D17" s="6" t="n">
+        <v>8.431079999999998</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>aten::_mps_convolution</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>50</v>
+      </c>
+      <c r="C18" s="6" t="n">
+        <v>4.461662999999997</v>
+      </c>
+      <c r="D18" s="6" t="n">
+        <v>4.548296000000004</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>profiled_model_inference</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>10</v>
+      </c>
+      <c r="C19" s="6" t="n">
+        <v>2.337674000000029</v>
+      </c>
+      <c r="D19" s="6" t="n">
+        <v>17.313168</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>aten::relu_</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>50</v>
+      </c>
+      <c r="C20" s="6" t="n">
+        <v>0.4901679999999928</v>
+      </c>
+      <c r="D20" s="6" t="n">
+        <v>0.4901679999999928</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>aten::linear</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>10</v>
+      </c>
+      <c r="C21" s="6" t="n">
+        <v>0.4623360000000002</v>
+      </c>
+      <c r="D21" s="6" t="n">
+        <v>0.5657930000000024</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>aten::empty</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>280</v>
+      </c>
+      <c r="C22" s="6" t="n">
+        <v>0.3170470000000143</v>
+      </c>
+      <c r="D22" s="6" t="n">
+        <v>0.3170470000000143</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>aten::_convolution</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>50</v>
+      </c>
+      <c r="C23" s="6" t="n">
+        <v>0.1572009999999959</v>
+      </c>
+      <c r="D23" s="6" t="n">
+        <v>4.705496999999999</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>aten::_batch_norm_impl_index</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>50</v>
+      </c>
+      <c r="C24" s="6" t="n">
+        <v>0.1351709999999975</v>
+      </c>
+      <c r="D24" s="6" t="n">
+        <v>8.60783099999999</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>aten::mean</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>10</v>
+      </c>
+      <c r="C25" s="6" t="n">
+        <v>0.1326250000000018</v>
+      </c>
+      <c r="D25" s="6" t="n">
+        <v>0.1326250000000018</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>aten::max_pool2d</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>20</v>
+      </c>
+      <c r="C26" s="6" t="n">
+        <v>0.1081629999999909</v>
+      </c>
+      <c r="D26" s="6" t="n">
+        <v>0.162041999999989</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>aten::batch_norm</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>50</v>
+      </c>
+      <c r="C27" s="6" t="n">
+        <v>0.1012080000000037</v>
+      </c>
+      <c r="D27" s="6" t="n">
+        <v>8.709038999999994</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>aten::convolution</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>50</v>
+      </c>
+      <c r="C28" s="6" t="n">
+        <v>0.09224899999999615</v>
+      </c>
+      <c r="D28" s="6" t="n">
+        <v>4.797745999999996</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A15:M15"/>
+    <mergeCell ref="A2:M2"/>
+    <mergeCell ref="A11:M11"/>
+    <mergeCell ref="A1:M1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="23" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>CUDA vs Apple Metal / MPS — profiling comparison</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>CUDA values are the existing Tesla T4 / Google Colab baseline. MPS values are the latest local profile. Different machines and PyTorch versions make this a practical hardware comparison, not a controlled experiment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Model-only inference (inputs already on the accelerator)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Batch</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>CUDA mean ms</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>MPS mean ms</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>CUDA faster (mean ×)</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>CUDA p50 ms</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>MPS p50 ms</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>CUDA faster (p50 ×)</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>MPS end-to-end mean ms</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>MPS end-to-end img/s</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>0.646</v>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>1.214466894889483</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>1.879979713451212</v>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>0.638</v>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>1.077749984688126</v>
+      </c>
+      <c r="G6" s="6" t="n">
+        <v>1.689263298884209</v>
+      </c>
+      <c r="H6" s="6" t="n">
+        <v>2.516636250220472</v>
+      </c>
+      <c r="I6" s="6" t="n">
+        <v>397.3557958216624</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>8</v>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>0.905</v>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>1.50210502644768</v>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>1.659784559610696</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>1.025</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>1.448062495910563</v>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>1.412743898449329</v>
+      </c>
+      <c r="H7" s="6" t="n">
+        <v>3.083426739467541</v>
+      </c>
+      <c r="I7" s="6" t="n">
+        <v>2594.515996634794</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>32</v>
+      </c>
+      <c r="B8" s="6" t="n">
+        <v>1.79</v>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>5.689578560413793</v>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>3.178535508611057</v>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>1.779</v>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>4.981688005500473</v>
+      </c>
+      <c r="G8" s="6" t="n">
+        <v>2.800274314502796</v>
+      </c>
+      <c r="H8" s="6" t="n">
+        <v>8.676391015033005</v>
+      </c>
+      <c r="I8" s="6" t="n">
+        <v>3688.169417970644</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>128</v>
+      </c>
+      <c r="B9" s="6" t="n">
+        <v>6.67</v>
+      </c>
+      <c r="C9" s="6" t="n">
+        <v>14.09337812292506</v>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>2.1129502433171</v>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>6.64</v>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>14.00985399959609</v>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>2.109917771023508</v>
+      </c>
+      <c r="H9" s="6" t="n">
+        <v>14.51253311970504</v>
+      </c>
+      <c r="I9" s="6" t="n">
+        <v>8819.962644991472</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Training step (batch 128)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Mean ms</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>p50 ms</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>p95 ms</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Images/s</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>CUDA faster (mean ×)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>CUDA / Tesla T4</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="n">
+        <v>22.11551510004938</v>
+      </c>
+      <c r="C13" s="6" t="n">
+        <v>22.12051499986956</v>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>22.3654986001975</v>
+      </c>
+      <c r="E13" s="6" t="n">
+        <v>5787.791937964593</v>
+      </c>
+      <c r="F13" s="6" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>MPS / Apple Metal</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="n">
+        <v>43.31685922166798</v>
+      </c>
+      <c r="C14" s="6" t="n">
+        <v>42.16202101088129</v>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>49.91002936294535</v>
+      </c>
+      <c r="E14" s="6" t="n">
+        <v>2954.969549961549</v>
+      </c>
+      <c r="F14" s="6" t="n">
+        <v>1.958663817039978</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>Kernel timing interpretation</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>CUDA can report current-stream GPU elapsed time through CUDA events. PyTorch has no matching MPS event timer; the MPS values use host monotonic time bracketed by torch.mps.synchronize(), which includes completed queued Metal work. For individual Metal kernels, record profile_cifar10.py --mps-signposts with Xcode Instruments → Metal System Trace.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A11:I11"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A17:I17"/>
+    <mergeCell ref="A4:I4"/>
+    <mergeCell ref="A16:I16"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>